<commit_message>
docs: synchronize REST documentation with actual implementation
</commit_message>
<xml_diff>
--- a/REST.xlsx
+++ b/REST.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\jakob\g1t2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC19F153-0902-40B5-B929-27246774A6A2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E637B31-3B1A-456F-8EE4-D8EF48431792}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="8040" windowHeight="9705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11805" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Frontend &lt;-&gt; Backend" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="181">
   <si>
     <t>URI-Template</t>
   </si>
@@ -405,9 +405,6 @@
     <t>Collection&lt;CartItemDTO&gt;</t>
   </si>
   <si>
-    <t>Collection&lt;OrderItemDTO&gt;</t>
-  </si>
-  <si>
     <t>productName</t>
   </si>
   <si>
@@ -450,21 +447,12 @@
     <t>OrderStatus</t>
   </si>
   <si>
-    <t>priceAtOrder</t>
-  </si>
-  <si>
     <t>phone</t>
   </si>
   <si>
     <t>discount</t>
   </si>
   <si>
-    <t>timestamp</t>
-  </si>
-  <si>
-    <t>discountAtOrder</t>
-  </si>
-  <si>
     <t>enabled</t>
   </si>
   <si>
@@ -552,7 +540,31 @@
     <t>UserxRole[]</t>
   </si>
   <si>
-    <t>CartDTO</t>
+    <t>CheckoutRequestDTO</t>
+  </si>
+  <si>
+    <t>orderDate</t>
+  </si>
+  <si>
+    <t>List&lt;OrderItemDTO&gt;</t>
+  </si>
+  <si>
+    <t>shippingName</t>
+  </si>
+  <si>
+    <t>paymentMethod</t>
+  </si>
+  <si>
+    <t>quantity</t>
+  </si>
+  <si>
+    <t>int</t>
+  </si>
+  <si>
+    <t>priceAtOPurchase</t>
+  </si>
+  <si>
+    <t>discountAtPurchase</t>
   </si>
 </sst>
 </file>
@@ -873,23 +885,23 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="12" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1839,10 +1851,10 @@
       </c>
       <c r="E27" s="12"/>
       <c r="F27" s="11" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="H27" s="11" t="s">
         <v>89</v>
@@ -1908,52 +1920,54 @@
     <col min="28" max="28" width="20.5703125" customWidth="1"/>
     <col min="29" max="31" width="14.140625" customWidth="1"/>
     <col min="32" max="32" width="22" customWidth="1"/>
-    <col min="33" max="66" width="14.140625" customWidth="1"/>
+    <col min="33" max="33" width="14.140625" customWidth="1"/>
+    <col min="34" max="34" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="35" max="66" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:66" ht="15.75" customHeight="1">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="35" t="s">
         <v>92</v>
       </c>
       <c r="B1" s="32"/>
-      <c r="D1" s="31" t="s">
+      <c r="D1" s="35" t="s">
         <v>93</v>
       </c>
       <c r="E1" s="32"/>
-      <c r="G1" s="31" t="s">
+      <c r="G1" s="35" t="s">
         <v>94</v>
       </c>
       <c r="H1" s="32"/>
-      <c r="J1" s="31" t="s">
+      <c r="J1" s="35" t="s">
         <v>95</v>
       </c>
       <c r="K1" s="32"/>
-      <c r="M1" s="31" t="s">
+      <c r="M1" s="35" t="s">
         <v>96</v>
       </c>
       <c r="N1" s="32"/>
-      <c r="P1" s="31" t="s">
+      <c r="P1" s="35" t="s">
         <v>97</v>
       </c>
       <c r="Q1" s="32"/>
-      <c r="V1" s="31" t="s">
+      <c r="V1" s="35" t="s">
         <v>98</v>
       </c>
       <c r="W1" s="32"/>
-      <c r="Y1" s="31" t="s">
+      <c r="Y1" s="35" t="s">
         <v>99</v>
       </c>
       <c r="Z1" s="32"/>
-      <c r="AB1" s="31" t="s">
+      <c r="AB1" s="35" t="s">
         <v>100</v>
       </c>
       <c r="AC1" s="32"/>
-      <c r="AE1" s="33" t="s">
+      <c r="AE1" s="37" t="s">
         <v>101</v>
       </c>
       <c r="AF1" s="32"/>
       <c r="AG1" s="15"/>
-      <c r="AH1" s="33" t="s">
+      <c r="AH1" s="37" t="s">
         <v>102</v>
       </c>
       <c r="AI1" s="32"/>
@@ -2026,7 +2040,7 @@
       <c r="Q2" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="S2" s="31" t="s">
+      <c r="S2" s="35" t="s">
         <v>105</v>
       </c>
       <c r="T2" s="32"/>
@@ -2093,7 +2107,7 @@
       <c r="BM2" s="16"/>
       <c r="BN2" s="16"/>
     </row>
-    <row r="3" spans="1:66">
+    <row r="3" spans="1:66" ht="15">
       <c r="A3" s="19" t="s">
         <v>106</v>
       </c>
@@ -2161,10 +2175,10 @@
         <v>107</v>
       </c>
       <c r="AG3" s="15"/>
-      <c r="AH3" s="22" t="s">
-        <v>106</v>
-      </c>
-      <c r="AI3" s="22" t="s">
+      <c r="AH3" s="24" t="s">
+        <v>110</v>
+      </c>
+      <c r="AI3" s="24" t="s">
         <v>107</v>
       </c>
       <c r="AJ3" s="23"/>
@@ -2199,7 +2213,7 @@
       <c r="BM3" s="23"/>
       <c r="BN3" s="23"/>
     </row>
-    <row r="4" spans="1:66">
+    <row r="4" spans="1:66" ht="12.75">
       <c r="A4" s="19" t="s">
         <v>111</v>
       </c>
@@ -2255,17 +2269,17 @@
         <v>118</v>
       </c>
       <c r="AE4" s="24" t="s">
-        <v>115</v>
+        <v>173</v>
       </c>
       <c r="AF4" s="24" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="AG4" s="15"/>
       <c r="AH4" s="24" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="AI4" s="24" t="s">
-        <v>107</v>
+        <v>36</v>
       </c>
       <c r="AJ4" s="23"/>
       <c r="AK4" s="23"/>
@@ -2299,7 +2313,7 @@
       <c r="BM4" s="23"/>
       <c r="BN4" s="23"/>
     </row>
-    <row r="5" spans="1:66">
+    <row r="5" spans="1:66" ht="12.75">
       <c r="A5" s="19" t="s">
         <v>119</v>
       </c>
@@ -2351,17 +2365,17 @@
       <c r="AB5" s="23"/>
       <c r="AC5" s="23"/>
       <c r="AE5" s="24" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="AF5" s="24" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="AG5" s="15"/>
       <c r="AH5" s="24" t="s">
-        <v>128</v>
+        <v>177</v>
       </c>
       <c r="AI5" s="24" t="s">
-        <v>36</v>
+        <v>178</v>
       </c>
       <c r="AJ5" s="23"/>
       <c r="AK5" s="23"/>
@@ -2397,44 +2411,44 @@
     </row>
     <row r="6" spans="1:66" ht="15.75" customHeight="1">
       <c r="A6" s="19" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B6" s="19" t="s">
         <v>107</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E6" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="G6" s="31" t="s">
-        <v>131</v>
+      <c r="G6" s="35" t="s">
+        <v>130</v>
       </c>
       <c r="H6" s="32"/>
       <c r="J6" s="21" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K6" s="21" t="s">
         <v>36</v>
       </c>
       <c r="M6" s="25" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="N6" s="25" t="s">
         <v>36</v>
       </c>
       <c r="P6" s="21" t="s">
+        <v>132</v>
+      </c>
+      <c r="Q6" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="Q6" s="21" t="s">
-        <v>134</v>
-      </c>
       <c r="S6" s="21" t="s">
+        <v>132</v>
+      </c>
+      <c r="T6" s="21" t="s">
         <v>133</v>
-      </c>
-      <c r="T6" s="21" t="s">
-        <v>134</v>
       </c>
       <c r="V6" s="23"/>
       <c r="W6" s="23"/>
@@ -2447,17 +2461,17 @@
       <c r="AB6" s="23"/>
       <c r="AC6" s="23"/>
       <c r="AE6" s="24" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="AF6" s="24" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AG6" s="15"/>
       <c r="AH6" s="24" t="s">
-        <v>117</v>
+        <v>179</v>
       </c>
       <c r="AI6" s="24" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="AJ6" s="23"/>
       <c r="AK6" s="23"/>
@@ -2491,15 +2505,15 @@
       <c r="BM6" s="23"/>
       <c r="BN6" s="23"/>
     </row>
-    <row r="7" spans="1:66">
+    <row r="7" spans="1:66" ht="15">
       <c r="A7" s="19" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B7" s="19" t="s">
         <v>120</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E7" s="19" t="s">
         <v>36</v>
@@ -2511,7 +2525,7 @@
         <v>104</v>
       </c>
       <c r="J7" s="21" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K7" s="21" t="s">
         <v>120</v>
@@ -2519,32 +2533,32 @@
       <c r="M7" s="26"/>
       <c r="N7" s="26"/>
       <c r="P7" s="21" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="Q7" s="21" t="s">
         <v>107</v>
       </c>
       <c r="S7" s="21" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="T7" s="21" t="s">
         <v>107</v>
       </c>
       <c r="AE7" s="24" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="AF7" s="24" t="s">
-        <v>141</v>
+        <v>174</v>
       </c>
       <c r="AG7" s="15"/>
       <c r="AH7" s="24" t="s">
-        <v>142</v>
+        <v>180</v>
       </c>
       <c r="AI7" s="24" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="8" spans="1:66">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8" spans="1:66" ht="12.75">
       <c r="A8" s="19" t="s">
         <v>108</v>
       </c>
@@ -2552,7 +2566,7 @@
         <v>36</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E8" s="19" t="s">
         <v>36</v>
@@ -2564,32 +2578,26 @@
         <v>36</v>
       </c>
       <c r="P8" s="21" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q8" s="21" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="S8" s="21" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T8" s="21" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AE8" s="24" t="s">
-        <v>145</v>
+        <v>175</v>
       </c>
       <c r="AF8" s="24" t="s">
-        <v>120</v>
+        <v>36</v>
       </c>
       <c r="AG8" s="15"/>
-      <c r="AH8" s="24" t="s">
-        <v>146</v>
-      </c>
-      <c r="AI8" s="24" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="9" spans="1:66">
+    </row>
+    <row r="9" spans="1:66" ht="12.75">
       <c r="A9" s="19" t="s">
         <v>121</v>
       </c>
@@ -2597,10 +2605,10 @@
         <v>36</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="G9" s="19" t="s">
         <v>112</v>
@@ -2609,35 +2617,39 @@
         <v>36</v>
       </c>
       <c r="P9" s="21" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="Q9" s="21" t="s">
         <v>36</v>
       </c>
       <c r="S9" s="21" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="T9" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="AE9" s="15"/>
-      <c r="AF9" s="15"/>
+      <c r="AE9" s="24" t="s">
+        <v>176</v>
+      </c>
+      <c r="AF9" s="24" t="s">
+        <v>36</v>
+      </c>
       <c r="AG9" s="15"/>
       <c r="AH9" s="15"/>
       <c r="AI9" s="15"/>
     </row>
-    <row r="10" spans="1:66">
+    <row r="10" spans="1:66" ht="12.75">
       <c r="A10" s="19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B10" s="19" t="s">
         <v>36</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="AE10" s="15"/>
       <c r="AF10" s="15"/>
@@ -2645,9 +2657,9 @@
       <c r="AH10" s="15"/>
       <c r="AI10" s="15"/>
     </row>
-    <row r="11" spans="1:66">
+    <row r="11" spans="1:66" ht="12.75">
       <c r="A11" s="19" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B11" s="19" t="s">
         <v>36</v>
@@ -2658,9 +2670,9 @@
       <c r="AH11" s="15"/>
       <c r="AI11" s="15"/>
     </row>
-    <row r="12" spans="1:66">
+    <row r="12" spans="1:66" ht="12.75">
       <c r="A12" s="19" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B12" s="19" t="s">
         <v>36</v>
@@ -2671,12 +2683,12 @@
       <c r="AH12" s="15"/>
       <c r="AI12" s="15"/>
     </row>
-    <row r="13" spans="1:66">
+    <row r="13" spans="1:66" ht="12.75">
       <c r="A13" s="19" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="AE13" s="15"/>
       <c r="AF13" s="15"/>
@@ -2684,12 +2696,12 @@
       <c r="AH13" s="15"/>
       <c r="AI13" s="15"/>
     </row>
-    <row r="14" spans="1:66">
+    <row r="14" spans="1:66" ht="12.75">
       <c r="A14" s="19" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="AE14" s="15"/>
       <c r="AF14" s="15"/>
@@ -2697,14 +2709,14 @@
       <c r="AH14" s="15"/>
       <c r="AI14" s="15"/>
     </row>
-    <row r="15" spans="1:66">
+    <row r="15" spans="1:66" ht="12.75">
       <c r="AE15" s="15"/>
       <c r="AF15" s="15"/>
       <c r="AG15" s="15"/>
       <c r="AH15" s="15"/>
       <c r="AI15" s="15"/>
     </row>
-    <row r="16" spans="1:66">
+    <row r="16" spans="1:66" ht="12.75">
       <c r="AE16" s="15"/>
       <c r="AF16" s="15"/>
       <c r="AG16" s="15"/>
@@ -2712,39 +2724,39 @@
       <c r="AI16" s="15"/>
     </row>
     <row r="17" spans="1:35" ht="15.75" customHeight="1">
-      <c r="A17" s="34" t="s">
+      <c r="A17" s="31" t="s">
+        <v>148</v>
+      </c>
+      <c r="B17" s="32"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="34"/>
+      <c r="G17" s="31" t="s">
+        <v>149</v>
+      </c>
+      <c r="H17" s="32"/>
+      <c r="J17" s="31" t="s">
+        <v>150</v>
+      </c>
+      <c r="K17" s="32"/>
+      <c r="P17" s="31" t="s">
+        <v>151</v>
+      </c>
+      <c r="Q17" s="32"/>
+      <c r="V17" s="31" t="s">
         <v>152</v>
       </c>
-      <c r="B17" s="32"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="37"/>
-      <c r="G17" s="34" t="s">
+      <c r="W17" s="32"/>
+      <c r="Y17" s="31" t="s">
         <v>153</v>
       </c>
-      <c r="H17" s="32"/>
-      <c r="J17" s="34" t="s">
+      <c r="Z17" s="32"/>
+      <c r="AE17" s="36" t="s">
         <v>154</v>
-      </c>
-      <c r="K17" s="32"/>
-      <c r="P17" s="34" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q17" s="32"/>
-      <c r="V17" s="34" t="s">
-        <v>156</v>
-      </c>
-      <c r="W17" s="32"/>
-      <c r="Y17" s="34" t="s">
-        <v>157</v>
-      </c>
-      <c r="Z17" s="32"/>
-      <c r="AE17" s="35" t="s">
-        <v>158</v>
       </c>
       <c r="AF17" s="32"/>
       <c r="AG17" s="15"/>
-      <c r="AH17" s="35" t="s">
-        <v>159</v>
+      <c r="AH17" s="36" t="s">
+        <v>155</v>
       </c>
       <c r="AI17" s="32"/>
     </row>
@@ -2779,8 +2791,8 @@
       <c r="Q18" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="S18" s="34" t="s">
-        <v>160</v>
+      <c r="S18" s="31" t="s">
+        <v>156</v>
       </c>
       <c r="T18" s="32"/>
       <c r="V18" s="17" t="s">
@@ -2809,36 +2821,36 @@
         <v>104</v>
       </c>
     </row>
-    <row r="19" spans="1:35">
+    <row r="19" spans="1:35" ht="15">
       <c r="A19" s="19" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="D19" s="28" t="s">
         <v>108</v>
       </c>
       <c r="E19" s="28" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="G19" s="19" t="s">
         <v>108</v>
       </c>
       <c r="H19" s="19" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="J19" s="20" t="s">
         <v>106</v>
       </c>
       <c r="K19" s="20" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="P19" s="20" t="s">
         <v>106</v>
       </c>
       <c r="Q19" s="20" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="S19" s="17" t="s">
         <v>103</v>
@@ -2850,52 +2862,52 @@
         <v>106</v>
       </c>
       <c r="W19" s="20" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="Y19" s="20" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="Z19" s="20" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="AE19" s="22" t="s">
         <v>106</v>
       </c>
       <c r="AF19" s="22" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="AG19" s="15"/>
-      <c r="AH19" s="22" t="s">
-        <v>106</v>
+      <c r="AH19" s="24" t="s">
+        <v>110</v>
       </c>
       <c r="AI19" s="22" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="20" spans="1:35">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="20" spans="1:35" ht="12.75">
       <c r="A20" s="19" t="s">
         <v>108</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="D20" s="28" t="s">
         <v>112</v>
       </c>
       <c r="E20" s="28" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="G20" s="19" t="s">
         <v>112</v>
       </c>
       <c r="H20" s="19" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="J20" s="21" t="s">
         <v>113</v>
       </c>
       <c r="K20" s="21" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="P20" s="21" t="s">
         <v>114</v>
@@ -2913,34 +2925,34 @@
         <v>115</v>
       </c>
       <c r="W20" s="21" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="Y20" s="21" t="s">
         <v>116</v>
       </c>
       <c r="Z20" s="20" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="AE20" s="24" t="s">
-        <v>115</v>
+        <v>173</v>
       </c>
       <c r="AF20" s="24" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="AG20" s="15"/>
       <c r="AH20" s="24" t="s">
-        <v>110</v>
-      </c>
-      <c r="AI20" s="22" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="21" spans="1:35">
+        <v>127</v>
+      </c>
+      <c r="AI20" s="24" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="21" spans="1:35" ht="12.75">
       <c r="A21" s="19" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="D21" s="29"/>
       <c r="E21" s="29"/>
@@ -2966,54 +2978,54 @@
         <v>125</v>
       </c>
       <c r="W21" s="21" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="Y21" s="21" t="s">
         <v>110</v>
       </c>
       <c r="Z21" s="20" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="AE21" s="24" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="AF21" s="24" t="s">
-        <v>167</v>
+        <v>140</v>
       </c>
       <c r="AG21" s="15"/>
       <c r="AH21" s="24" t="s">
-        <v>128</v>
-      </c>
-      <c r="AI21" s="24" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="22" spans="1:35">
+        <v>177</v>
+      </c>
+      <c r="AI21" s="22" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="22" spans="1:35" ht="12.75">
       <c r="A22" s="19" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="D22" s="29"/>
       <c r="E22" s="29"/>
       <c r="J22" s="21" t="s">
+        <v>131</v>
+      </c>
+      <c r="K22" s="21" t="s">
+        <v>159</v>
+      </c>
+      <c r="P22" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="K22" s="21" t="s">
-        <v>163</v>
-      </c>
-      <c r="P22" s="21" t="s">
-        <v>133</v>
-      </c>
       <c r="Q22" s="20" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="S22" s="21" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="T22" s="20" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="V22" s="30"/>
       <c r="W22" s="30"/>
@@ -3021,75 +3033,75 @@
         <v>117</v>
       </c>
       <c r="Z22" s="20" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="AE22" s="24" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="AF22" s="24" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="AG22" s="15"/>
       <c r="AH22" s="24" t="s">
-        <v>117</v>
-      </c>
-      <c r="AI22" s="22" t="s">
-        <v>162</v>
+        <v>179</v>
+      </c>
+      <c r="AI22" s="24" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="23" spans="1:35" ht="15.75" customHeight="1">
       <c r="A23" s="19" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>165</v>
-      </c>
-      <c r="D23" s="36"/>
-      <c r="E23" s="37"/>
-      <c r="G23" s="34" t="s">
-        <v>171</v>
+        <v>161</v>
+      </c>
+      <c r="D23" s="33"/>
+      <c r="E23" s="34"/>
+      <c r="G23" s="31" t="s">
+        <v>167</v>
       </c>
       <c r="H23" s="32"/>
       <c r="J23" s="21" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K23" s="21" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="M23" s="30"/>
       <c r="N23" s="30"/>
       <c r="P23" s="21" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="Q23" s="20" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="S23" s="21" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="T23" s="20" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="AE23" s="24" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="AF23" s="24" t="s">
         <v>163</v>
       </c>
       <c r="AG23" s="15"/>
       <c r="AH23" s="24" t="s">
-        <v>142</v>
+        <v>180</v>
       </c>
       <c r="AI23" s="24" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="24" spans="1:35">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="24" spans="1:35" ht="15">
       <c r="A24" s="19" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="D24" s="27" t="s">
         <v>103</v>
@@ -3104,124 +3116,118 @@
         <v>104</v>
       </c>
       <c r="P24" s="21" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Q24" s="20" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="S24" s="21" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="T24" s="20" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="AE24" s="24" t="s">
-        <v>145</v>
+        <v>175</v>
       </c>
       <c r="AF24" s="24" t="s">
-        <v>172</v>
+        <v>159</v>
       </c>
       <c r="AG24" s="15"/>
-      <c r="AH24" s="24" t="s">
-        <v>146</v>
-      </c>
-      <c r="AI24" s="24" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="25" spans="1:35">
+    </row>
+    <row r="25" spans="1:35" ht="12.75">
       <c r="A25" s="19" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="D25" s="28" t="s">
         <v>109</v>
       </c>
       <c r="E25" s="28" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="G25" s="19" t="s">
         <v>109</v>
       </c>
       <c r="H25" s="19" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="P25" s="21" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="Q25" s="21" t="s">
         <v>36</v>
       </c>
       <c r="S25" s="21" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="T25" s="21" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="26" spans="1:35">
+      <c r="AE25" s="24" t="s">
+        <v>176</v>
+      </c>
+      <c r="AF25" s="24" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="26" spans="1:35" ht="12.75">
       <c r="A26" s="19" t="s">
         <v>121</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="27" spans="1:35">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="27" spans="1:35" ht="12.75">
       <c r="A27" s="19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="28" spans="1:35">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="28" spans="1:35" ht="12.75">
       <c r="A28" s="19" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="29" spans="1:35">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="29" spans="1:35" ht="12.75">
       <c r="A29" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="B29" s="19" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="30" spans="1:35" ht="12.75">
+      <c r="A30" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="B29" s="19" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="30" spans="1:35">
-      <c r="A30" s="19" t="s">
-        <v>147</v>
-      </c>
       <c r="B30" s="19" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="31" spans="1:35">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="31" spans="1:35" ht="12.75">
       <c r="A31" s="19" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="P17:Q17"/>
-    <mergeCell ref="S18:T18"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="G23:H23"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="S2:T2"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="P1:Q1"/>
     <mergeCell ref="V17:W17"/>
     <mergeCell ref="Y17:Z17"/>
     <mergeCell ref="AE17:AF17"/>
@@ -3230,12 +3236,18 @@
     <mergeCell ref="AB1:AC1"/>
     <mergeCell ref="AE1:AF1"/>
     <mergeCell ref="AH1:AI1"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="M1:N1"/>
-    <mergeCell ref="P1:Q1"/>
     <mergeCell ref="V1:W1"/>
+    <mergeCell ref="S18:T18"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="S2:T2"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="P17:Q17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>